<commit_message>
IMPORTRANGE listos para Google Sheets: bloques vacíos salvo la primera celda
arreglar_dummy ahora también vacía en el XML las celdas COMPUTED_VALUE de
cada bloque (si tienen algo, Sheets no expande el resultado y da #REF!).
Los demás valores calculados quedan guardados. Regenerados los 6 Excel;
Manuales y Carros toman además las piezas por hoja vigentes del corte.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E33CYXtZ2f33D1RjoRdR65
</commit_message>
<xml_diff>
--- a/salida/Analisis_alternativas_corte_chapa.xlsx
+++ b/salida/Analisis_alternativas_corte_chapa.xlsx
@@ -2537,11 +2537,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="23936482"/>
-        <c:axId val="83372265"/>
+        <c:axId val="45722473"/>
+        <c:axId val="80739218"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="23936482"/>
+        <c:axId val="45722473"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2573,7 +2573,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83372265"/>
+        <c:crossAx val="80739218"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2581,7 +2581,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="83372265"/>
+        <c:axId val="80739218"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -2658,7 +2658,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="23936482"/>
+        <c:crossAx val="45722473"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3069,42 +3069,15 @@
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(Links!$B$4,""Indexado Dim Técnico!B3:K10"")"),4178.736543)</f>
         <v>4178.736543</v>
       </c>
-      <c r="D11" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5997.303977)</f>
-        <v>5997.303977</v>
-      </c>
-      <c r="E11" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),6851.747758)</f>
-        <v>6851.747758</v>
-      </c>
-      <c r="F11" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),8467.135549)</f>
-        <v>8467.135549</v>
-      </c>
-      <c r="G11" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),12680.63271)</f>
-        <v>12680.63271</v>
-      </c>
-      <c r="H11" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),15620.25307)</f>
-        <v>15620.25307</v>
-      </c>
-      <c r="I11" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),20332.55326)</f>
-        <v>20332.55326</v>
-      </c>
-      <c r="J11" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),25132.07848)</f>
-        <v>25132.07848</v>
-      </c>
-      <c r="K11" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),28573.33614)</f>
-        <v>28573.33614</v>
-      </c>
-      <c r="L11" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),32072.63913)</f>
-        <v>32072.63913</v>
-      </c>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="9"/>
+      <c r="L11" s="9"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
@@ -3113,46 +3086,16 @@
       <c r="B12" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),295.0303572)</f>
-        <v>295.0303572</v>
-      </c>
-      <c r="D12" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),709.7274503)</f>
-        <v>709.7274503</v>
-      </c>
-      <c r="E12" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),986.8680576)</f>
-        <v>986.8680576</v>
-      </c>
-      <c r="F12" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1500.638174)</f>
-        <v>1500.638174</v>
-      </c>
-      <c r="G12" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2312.627726)</f>
-        <v>2312.627726</v>
-      </c>
-      <c r="H12" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3252.869887)</f>
-        <v>3252.869887</v>
-      </c>
-      <c r="I12" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4102.315524)</f>
-        <v>4102.315524</v>
-      </c>
-      <c r="J12" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5104.306587)</f>
-        <v>5104.306587</v>
-      </c>
-      <c r="K12" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),6195.186243)</f>
-        <v>6195.186243</v>
-      </c>
-      <c r="L12" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7424.858444)</f>
-        <v>7424.858444</v>
-      </c>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="9"/>
+      <c r="J12" s="9"/>
+      <c r="K12" s="9"/>
+      <c r="L12" s="9"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
@@ -3161,46 +3104,16 @@
       <c r="B13" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C13" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2255.773025)</f>
-        <v>2255.773025</v>
-      </c>
-      <c r="D13" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3846.978881)</f>
-        <v>3846.978881</v>
-      </c>
-      <c r="E13" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5093.537591)</f>
-        <v>5093.537591</v>
-      </c>
-      <c r="F13" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),6823.115313)</f>
-        <v>6823.115313</v>
-      </c>
-      <c r="G13" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),10819.30694)</f>
-        <v>10819.30694</v>
-      </c>
-      <c r="H13" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),14605.96411)</f>
-        <v>14605.96411</v>
-      </c>
-      <c r="I13" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),18877.75984)</f>
-        <v>18877.75984</v>
-      </c>
-      <c r="J13" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),23368.18637)</f>
-        <v>23368.18637</v>
-      </c>
-      <c r="K13" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),26967.72455)</f>
-        <v>26967.72455</v>
-      </c>
-      <c r="L13" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),30750.77872)</f>
-        <v>30750.77872</v>
-      </c>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="9"/>
+      <c r="L13" s="9"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
@@ -3209,46 +3122,16 @@
       <c r="B14" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C14" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),91.83318153)</f>
-        <v>91.83318153</v>
-      </c>
-      <c r="D14" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),177.2472967)</f>
-        <v>177.2472967</v>
-      </c>
-      <c r="E14" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),252.9787798)</f>
-        <v>252.9787798</v>
-      </c>
-      <c r="F14" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),358.0204941)</f>
-        <v>358.0204941</v>
-      </c>
-      <c r="G14" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),602.7181519)</f>
-        <v>602.7181519</v>
-      </c>
-      <c r="H14" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),872.605032)</f>
-        <v>872.605032</v>
-      </c>
-      <c r="I14" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1127.160545)</f>
-        <v>1127.160545</v>
-      </c>
-      <c r="J14" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1395.444812)</f>
-        <v>1395.444812</v>
-      </c>
-      <c r="K14" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1612.350054)</f>
-        <v>1612.350054</v>
-      </c>
-      <c r="L14" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1840.848079)</f>
-        <v>1840.848079</v>
-      </c>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="9"/>
+      <c r="L14" s="9"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
@@ -3257,46 +3140,16 @@
       <c r="B15" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C15" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),34.05179136)</f>
-        <v>34.05179136</v>
-      </c>
-      <c r="D15" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),58.46214745)</f>
-        <v>58.46214745</v>
-      </c>
-      <c r="E15" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),75.20853998)</f>
-        <v>75.20853998</v>
-      </c>
-      <c r="F15" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),100.5298529)</f>
-        <v>100.5298529</v>
-      </c>
-      <c r="G15" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),155.8760035)</f>
-        <v>155.8760035</v>
-      </c>
-      <c r="H15" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),211.9344827)</f>
-        <v>211.9344827</v>
-      </c>
-      <c r="I15" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),272.6682332)</f>
-        <v>272.6682332</v>
-      </c>
-      <c r="J15" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),337.8486707)</f>
-        <v>337.8486707</v>
-      </c>
-      <c r="K15" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),393.6274156)</f>
-        <v>393.6274156</v>
-      </c>
-      <c r="L15" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),453.2705332)</f>
-        <v>453.2705332</v>
-      </c>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="9"/>
+      <c r="K15" s="9"/>
+      <c r="L15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
@@ -3305,46 +3158,16 @@
       <c r="B16" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C16" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),74.913941)</f>
-        <v>74.913941</v>
-      </c>
-      <c r="D16" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),128.6167244)</f>
-        <v>128.6167244</v>
-      </c>
-      <c r="E16" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),165.458788)</f>
-        <v>165.458788</v>
-      </c>
-      <c r="F16" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),221.1656765)</f>
-        <v>221.1656765</v>
-      </c>
-      <c r="G16" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),342.9272077)</f>
-        <v>342.9272077</v>
-      </c>
-      <c r="H16" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),466.255862)</f>
-        <v>466.255862</v>
-      </c>
-      <c r="I16" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),599.8701129)</f>
-        <v>599.8701129</v>
-      </c>
-      <c r="J16" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),743.2670756)</f>
-        <v>743.2670756</v>
-      </c>
-      <c r="K16" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),865.9803143)</f>
-        <v>865.9803143</v>
-      </c>
-      <c r="L16" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),997.1951731)</f>
-        <v>997.1951731</v>
-      </c>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
+      <c r="J16" s="9"/>
+      <c r="K16" s="9"/>
+      <c r="L16" s="9"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
@@ -3353,46 +3176,16 @@
       <c r="B17" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),16.34485985)</f>
-        <v>16.34485985</v>
-      </c>
-      <c r="D17" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),28.06183078)</f>
-        <v>28.06183078</v>
-      </c>
-      <c r="E17" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),36.10009919)</f>
-        <v>36.10009919</v>
-      </c>
-      <c r="F17" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),48.25432941)</f>
-        <v>48.25432941</v>
-      </c>
-      <c r="G17" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),74.82048167)</f>
-        <v>74.82048167</v>
-      </c>
-      <c r="H17" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),101.7285517)</f>
-        <v>101.7285517</v>
-      </c>
-      <c r="I17" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),130.8807519)</f>
-        <v>130.8807519</v>
-      </c>
-      <c r="J17" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),162.1673619)</f>
-        <v>162.1673619</v>
-      </c>
-      <c r="K17" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),188.9411595)</f>
-        <v>188.9411595</v>
-      </c>
-      <c r="L17" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),217.569856)</f>
-        <v>217.569856</v>
-      </c>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="9"/>
+      <c r="K17" s="9"/>
+      <c r="L17" s="9"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
@@ -3401,46 +3194,16 @@
       <c r="B18" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C18" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),10.89657324)</f>
-        <v>10.89657324</v>
-      </c>
-      <c r="D18" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),18.70788719)</f>
-        <v>18.70788719</v>
-      </c>
-      <c r="E18" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),24.06673279)</f>
-        <v>24.06673279</v>
-      </c>
-      <c r="F18" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),32.16955294)</f>
-        <v>32.16955294</v>
-      </c>
-      <c r="G18" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),49.88032112)</f>
-        <v>49.88032112</v>
-      </c>
-      <c r="H18" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),67.81903447)</f>
-        <v>67.81903447</v>
-      </c>
-      <c r="I18" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),87.25383461)</f>
-        <v>87.25383461</v>
-      </c>
-      <c r="J18" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),108.1115746)</f>
-        <v>108.1115746</v>
-      </c>
-      <c r="K18" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),125.960773)</f>
-        <v>125.960773</v>
-      </c>
-      <c r="L18" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),145.0465706)</f>
-        <v>145.0465706</v>
-      </c>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="9"/>
+      <c r="J18" s="9"/>
+      <c r="K18" s="9"/>
+      <c r="L18" s="9"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
@@ -3496,42 +3259,15 @@
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(Links!$B$4,""Indexado Dim Técnico!B15:K22"")"),0)</f>
         <v>0</v>
       </c>
-      <c r="D22" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="E22" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7662.4)</f>
-        <v>7662.4</v>
-      </c>
-      <c r="F22" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),26694.8)</f>
-        <v>26694.8</v>
-      </c>
-      <c r="G22" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),49434.8)</f>
-        <v>49434.8</v>
-      </c>
-      <c r="H22" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),71680.2)</f>
-        <v>71680.2</v>
-      </c>
-      <c r="I22" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),101340.6)</f>
-        <v>101340.6</v>
-      </c>
-      <c r="J22" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),131001)</f>
-        <v>131001</v>
-      </c>
-      <c r="K22" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),146819.8)</f>
-        <v>146819.8</v>
-      </c>
-      <c r="L22" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),170548)</f>
-        <v>170548</v>
-      </c>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
+      <c r="J22" s="9"/>
+      <c r="K22" s="9"/>
+      <c r="L22" s="9"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
@@ -3540,46 +3276,16 @@
       <c r="B23" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C23" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="D23" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="E23" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),299.6)</f>
-        <v>299.6</v>
-      </c>
-      <c r="F23" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1043.8)</f>
-        <v>1043.8</v>
-      </c>
-      <c r="G23" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1933)</f>
-        <v>1933</v>
-      </c>
-      <c r="H23" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2803)</f>
-        <v>2803</v>
-      </c>
-      <c r="I23" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3963)</f>
-        <v>3963</v>
-      </c>
-      <c r="J23" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5123)</f>
-        <v>5123</v>
-      </c>
-      <c r="K23" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5741.4)</f>
-        <v>5741.4</v>
-      </c>
-      <c r="L23" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),6669)</f>
-        <v>6669</v>
-      </c>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
+      <c r="I23" s="9"/>
+      <c r="J23" s="9"/>
+      <c r="K23" s="9"/>
+      <c r="L23" s="9"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
@@ -3588,46 +3294,16 @@
       <c r="B24" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C24" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="D24" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="E24" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1478.8)</f>
-        <v>1478.8</v>
-      </c>
-      <c r="F24" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5152)</f>
-        <v>5152</v>
-      </c>
-      <c r="G24" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),9540.8)</f>
-        <v>9540.8</v>
-      </c>
-      <c r="H24" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),13834.2)</f>
-        <v>13834.2</v>
-      </c>
-      <c r="I24" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),19558.6)</f>
-        <v>19558.6</v>
-      </c>
-      <c r="J24" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),25283)</f>
-        <v>25283</v>
-      </c>
-      <c r="K24" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),28335.8)</f>
-        <v>28335.8</v>
-      </c>
-      <c r="L24" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),32915)</f>
-        <v>32915</v>
-      </c>
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
+      <c r="I24" s="9"/>
+      <c r="J24" s="9"/>
+      <c r="K24" s="9"/>
+      <c r="L24" s="9"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
@@ -3636,46 +3312,16 @@
       <c r="B25" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C25" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="D25" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="E25" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),90.4)</f>
-        <v>90.4</v>
-      </c>
-      <c r="F25" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),315)</f>
-        <v>315</v>
-      </c>
-      <c r="G25" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),583.4)</f>
-        <v>583.4</v>
-      </c>
-      <c r="H25" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),845.8)</f>
-        <v>845.8</v>
-      </c>
-      <c r="I25" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1195.4)</f>
-        <v>1195.4</v>
-      </c>
-      <c r="J25" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1545)</f>
-        <v>1545</v>
-      </c>
-      <c r="K25" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1731.4)</f>
-        <v>1731.4</v>
-      </c>
-      <c r="L25" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2011)</f>
-        <v>2011</v>
-      </c>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
+      <c r="I25" s="9"/>
+      <c r="J25" s="9"/>
+      <c r="K25" s="9"/>
+      <c r="L25" s="9"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
@@ -3684,46 +3330,16 @@
       <c r="B26" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C26" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="D26" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="E26" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),14.4)</f>
-        <v>14.4</v>
-      </c>
-      <c r="F26" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),50.2)</f>
-        <v>50.2</v>
-      </c>
-      <c r="G26" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),93)</f>
-        <v>93</v>
-      </c>
-      <c r="H26" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),135)</f>
-        <v>135</v>
-      </c>
-      <c r="I26" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),191)</f>
-        <v>191</v>
-      </c>
-      <c r="J26" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),247)</f>
-        <v>247</v>
-      </c>
-      <c r="K26" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),277)</f>
-        <v>277</v>
-      </c>
-      <c r="L26" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),322)</f>
-        <v>322</v>
-      </c>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
+      <c r="I26" s="9"/>
+      <c r="J26" s="9"/>
+      <c r="K26" s="9"/>
+      <c r="L26" s="9"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
@@ -3732,46 +3348,16 @@
       <c r="B27" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C27" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="D27" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="E27" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),31.8)</f>
-        <v>31.8</v>
-      </c>
-      <c r="F27" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),110.8)</f>
-        <v>110.8</v>
-      </c>
-      <c r="G27" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),205.2)</f>
-        <v>205.2</v>
-      </c>
-      <c r="H27" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),297.6)</f>
-        <v>297.6</v>
-      </c>
-      <c r="I27" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),420.8)</f>
-        <v>420.8</v>
-      </c>
-      <c r="J27" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),544)</f>
-        <v>544</v>
-      </c>
-      <c r="K27" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),609.6)</f>
-        <v>609.6</v>
-      </c>
-      <c r="L27" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),708)</f>
-        <v>708</v>
-      </c>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
+      <c r="I27" s="9"/>
+      <c r="J27" s="9"/>
+      <c r="K27" s="9"/>
+      <c r="L27" s="9"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
@@ -3780,46 +3366,16 @@
       <c r="B28" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C28" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="D28" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="E28" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7)</f>
-        <v>7</v>
-      </c>
-      <c r="F28" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),24.4)</f>
-        <v>24.4</v>
-      </c>
-      <c r="G28" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),45.2)</f>
-        <v>45.2</v>
-      </c>
-      <c r="H28" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),65.4)</f>
-        <v>65.4</v>
-      </c>
-      <c r="I28" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),92.2)</f>
-        <v>92.2</v>
-      </c>
-      <c r="J28" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),119)</f>
-        <v>119</v>
-      </c>
-      <c r="K28" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),133.4)</f>
-        <v>133.4</v>
-      </c>
-      <c r="L28" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),155)</f>
-        <v>155</v>
-      </c>
+      <c r="C28" s="9"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
+      <c r="F28" s="9"/>
+      <c r="G28" s="9"/>
+      <c r="H28" s="9"/>
+      <c r="I28" s="9"/>
+      <c r="J28" s="9"/>
+      <c r="K28" s="9"/>
+      <c r="L28" s="9"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
@@ -3828,46 +3384,16 @@
       <c r="B29" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C29" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="D29" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="E29" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.6)</f>
-        <v>4.6</v>
-      </c>
-      <c r="F29" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),16)</f>
-        <v>16</v>
-      </c>
-      <c r="G29" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),29.6)</f>
-        <v>29.6</v>
-      </c>
-      <c r="H29" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),42.8)</f>
-        <v>42.8</v>
-      </c>
-      <c r="I29" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),60.4)</f>
-        <v>60.4</v>
-      </c>
-      <c r="J29" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),78)</f>
-        <v>78</v>
-      </c>
-      <c r="K29" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),87.6)</f>
-        <v>87.6</v>
-      </c>
-      <c r="L29" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),102)</f>
-        <v>102</v>
-      </c>
+      <c r="C29" s="9"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="9"/>
+      <c r="F29" s="9"/>
+      <c r="G29" s="9"/>
+      <c r="H29" s="9"/>
+      <c r="I29" s="9"/>
+      <c r="J29" s="9"/>
+      <c r="K29" s="9"/>
+      <c r="L29" s="9"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="s">
@@ -3923,42 +3449,15 @@
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(Links!$B$6,""sobrestock_sustitutos!B73:K76"")"),0)</f>
         <v>0</v>
       </c>
-      <c r="D33" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="E33" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="F33" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="G33" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="H33" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="I33" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="J33" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K33" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="L33" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+      <c r="I33" s="9"/>
+      <c r="J33" s="9"/>
+      <c r="K33" s="9"/>
+      <c r="L33" s="9"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
@@ -3967,46 +3466,16 @@
       <c r="B34" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C34" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2)</f>
-        <v>2</v>
-      </c>
-      <c r="D34" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.16)</f>
-        <v>5.16</v>
-      </c>
-      <c r="E34" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.56)</f>
-        <v>7.56</v>
-      </c>
-      <c r="F34" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),13.12)</f>
-        <v>13.12</v>
-      </c>
-      <c r="G34" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),13.08)</f>
-        <v>13.08</v>
-      </c>
-      <c r="H34" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),14.96)</f>
-        <v>14.96</v>
-      </c>
-      <c r="I34" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),13.92)</f>
-        <v>13.92</v>
-      </c>
-      <c r="J34" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),10.72)</f>
-        <v>10.72</v>
-      </c>
-      <c r="K34" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),10.2)</f>
-        <v>10.2</v>
-      </c>
-      <c r="L34" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),11.6)</f>
-        <v>11.6</v>
-      </c>
+      <c r="C34" s="9"/>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
+      <c r="I34" s="9"/>
+      <c r="J34" s="9"/>
+      <c r="K34" s="9"/>
+      <c r="L34" s="9"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
@@ -4015,46 +3484,16 @@
       <c r="B35" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C35" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),9)</f>
-        <v>9</v>
-      </c>
-      <c r="D35" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),27.72)</f>
-        <v>27.72</v>
-      </c>
-      <c r="E35" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),47.88)</f>
-        <v>47.88</v>
-      </c>
-      <c r="F35" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),78.48)</f>
-        <v>78.48</v>
-      </c>
-      <c r="G35" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),80.24)</f>
-        <v>80.24</v>
-      </c>
-      <c r="H35" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),89.68)</f>
-        <v>89.68</v>
-      </c>
-      <c r="I35" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),77.44)</f>
-        <v>77.44</v>
-      </c>
-      <c r="J35" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),65.76)</f>
-        <v>65.76</v>
-      </c>
-      <c r="K35" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),60.8)</f>
-        <v>60.8</v>
-      </c>
-      <c r="L35" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),64.2)</f>
-        <v>64.2</v>
-      </c>
+      <c r="C35" s="9"/>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
+      <c r="G35" s="9"/>
+      <c r="H35" s="9"/>
+      <c r="I35" s="9"/>
+      <c r="J35" s="9"/>
+      <c r="K35" s="9"/>
+      <c r="L35" s="9"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
@@ -4063,46 +3502,16 @@
       <c r="B36" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C36" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1)</f>
-        <v>1</v>
-      </c>
-      <c r="D36" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.08)</f>
-        <v>2.08</v>
-      </c>
-      <c r="E36" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.24)</f>
-        <v>3.24</v>
-      </c>
-      <c r="F36" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.48)</f>
-        <v>4.48</v>
-      </c>
-      <c r="G36" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.8)</f>
-        <v>4.8</v>
-      </c>
-      <c r="H36" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),6.12)</f>
-        <v>6.12</v>
-      </c>
-      <c r="I36" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.52)</f>
-        <v>4.52</v>
-      </c>
-      <c r="J36" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.76)</f>
-        <v>3.76</v>
-      </c>
-      <c r="K36" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.92)</f>
-        <v>3.92</v>
-      </c>
-      <c r="L36" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.08)</f>
-        <v>4.08</v>
-      </c>
+      <c r="C36" s="9"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
+      <c r="I36" s="9"/>
+      <c r="J36" s="9"/>
+      <c r="K36" s="9"/>
+      <c r="L36" s="9"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
@@ -4115,42 +3524,15 @@
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(Links!$B$6,""sobrestock_sustitutos!B86:K89"")"),1)</f>
         <v>1</v>
       </c>
-      <c r="D37" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.08)</f>
-        <v>0.08</v>
-      </c>
-      <c r="E37" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.08)</f>
-        <v>0.08</v>
-      </c>
-      <c r="F37" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.08)</f>
-        <v>1.08</v>
-      </c>
-      <c r="G37" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.16)</f>
-        <v>1.16</v>
-      </c>
-      <c r="H37" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.24)</f>
-        <v>1.24</v>
-      </c>
-      <c r="I37" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.32)</f>
-        <v>0.32</v>
-      </c>
-      <c r="J37" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.32)</f>
-        <v>0.32</v>
-      </c>
-      <c r="K37" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.32)</f>
-        <v>1.32</v>
-      </c>
-      <c r="L37" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.4)</f>
-        <v>0.4</v>
-      </c>
+      <c r="D37" s="9"/>
+      <c r="E37" s="9"/>
+      <c r="F37" s="9"/>
+      <c r="G37" s="9"/>
+      <c r="H37" s="9"/>
+      <c r="I37" s="9"/>
+      <c r="J37" s="9"/>
+      <c r="K37" s="9"/>
+      <c r="L37" s="9"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="s">
@@ -4159,46 +3541,16 @@
       <c r="B38" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C38" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1)</f>
-        <v>1</v>
-      </c>
-      <c r="D38" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.08)</f>
-        <v>0.08</v>
-      </c>
-      <c r="E38" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.08)</f>
-        <v>1.08</v>
-      </c>
-      <c r="F38" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.16)</f>
-        <v>2.16</v>
-      </c>
-      <c r="G38" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.32)</f>
-        <v>2.32</v>
-      </c>
-      <c r="H38" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.48)</f>
-        <v>1.48</v>
-      </c>
-      <c r="I38" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.56)</f>
-        <v>1.56</v>
-      </c>
-      <c r="J38" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.64)</f>
-        <v>1.64</v>
-      </c>
-      <c r="K38" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.72)</f>
-        <v>1.72</v>
-      </c>
-      <c r="L38" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.8)</f>
-        <v>0.8</v>
-      </c>
+      <c r="C38" s="9"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="9"/>
+      <c r="F38" s="9"/>
+      <c r="G38" s="9"/>
+      <c r="H38" s="9"/>
+      <c r="I38" s="9"/>
+      <c r="J38" s="9"/>
+      <c r="K38" s="9"/>
+      <c r="L38" s="9"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
@@ -4207,46 +3559,16 @@
       <c r="B39" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C39" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1)</f>
-        <v>1</v>
-      </c>
-      <c r="D39" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.08)</f>
-        <v>0.08</v>
-      </c>
-      <c r="E39" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.08)</f>
-        <v>0.08</v>
-      </c>
-      <c r="F39" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.08)</f>
-        <v>0.08</v>
-      </c>
-      <c r="G39" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.08)</f>
-        <v>1.08</v>
-      </c>
-      <c r="H39" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.16)</f>
-        <v>0.16</v>
-      </c>
-      <c r="I39" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.16)</f>
-        <v>0.16</v>
-      </c>
-      <c r="J39" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.16)</f>
-        <v>0.16</v>
-      </c>
-      <c r="K39" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.16)</f>
-        <v>1.16</v>
-      </c>
-      <c r="L39" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.24)</f>
-        <v>0.24</v>
-      </c>
+      <c r="C39" s="9"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="9"/>
+      <c r="F39" s="9"/>
+      <c r="G39" s="9"/>
+      <c r="H39" s="9"/>
+      <c r="I39" s="9"/>
+      <c r="J39" s="9"/>
+      <c r="K39" s="9"/>
+      <c r="L39" s="9"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
@@ -4255,46 +3577,16 @@
       <c r="B40" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C40" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1)</f>
-        <v>1</v>
-      </c>
-      <c r="D40" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.08)</f>
-        <v>0.08</v>
-      </c>
-      <c r="E40" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.08)</f>
-        <v>0.08</v>
-      </c>
-      <c r="F40" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.08)</f>
-        <v>0.08</v>
-      </c>
-      <c r="G40" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.08)</f>
-        <v>0.08</v>
-      </c>
-      <c r="H40" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.08)</f>
-        <v>0.08</v>
-      </c>
-      <c r="I40" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.08)</f>
-        <v>1.08</v>
-      </c>
-      <c r="J40" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.16)</f>
-        <v>0.16</v>
-      </c>
-      <c r="K40" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.16)</f>
-        <v>0.16</v>
-      </c>
-      <c r="L40" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.16)</f>
-        <v>0.16</v>
-      </c>
+      <c r="C40" s="9"/>
+      <c r="D40" s="9"/>
+      <c r="E40" s="9"/>
+      <c r="F40" s="9"/>
+      <c r="G40" s="9"/>
+      <c r="H40" s="9"/>
+      <c r="I40" s="9"/>
+      <c r="J40" s="9"/>
+      <c r="K40" s="9"/>
+      <c r="L40" s="9"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="8" t="s">
@@ -4350,42 +3642,15 @@
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(Links!$B$5,""sobrestock_sustitutos!B73:K76"")"),0)</f>
         <v>0</v>
       </c>
-      <c r="D44" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="E44" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="F44" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="G44" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="H44" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="I44" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="J44" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K44" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
-      <c r="L44" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0)</f>
-        <v>0</v>
-      </c>
+      <c r="D44" s="9"/>
+      <c r="E44" s="9"/>
+      <c r="F44" s="9"/>
+      <c r="G44" s="9"/>
+      <c r="H44" s="9"/>
+      <c r="I44" s="9"/>
+      <c r="J44" s="9"/>
+      <c r="K44" s="9"/>
+      <c r="L44" s="9"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="s">
@@ -4394,46 +3659,16 @@
       <c r="B45" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C45" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3)</f>
-        <v>3</v>
-      </c>
-      <c r="D45" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),9.24)</f>
-        <v>9.24</v>
-      </c>
-      <c r="E45" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),15.96)</f>
-        <v>15.96</v>
-      </c>
-      <c r="F45" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),24.16)</f>
-        <v>24.16</v>
-      </c>
-      <c r="G45" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),25.92)</f>
-        <v>25.92</v>
-      </c>
-      <c r="H45" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),28.68)</f>
-        <v>28.68</v>
-      </c>
-      <c r="I45" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),26.52)</f>
-        <v>26.52</v>
-      </c>
-      <c r="J45" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),21.04)</f>
-        <v>21.04</v>
-      </c>
-      <c r="K45" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),21)</f>
-        <v>21</v>
-      </c>
-      <c r="L45" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),20.88)</f>
-        <v>20.88</v>
-      </c>
+      <c r="C45" s="9"/>
+      <c r="D45" s="9"/>
+      <c r="E45" s="9"/>
+      <c r="F45" s="9"/>
+      <c r="G45" s="9"/>
+      <c r="H45" s="9"/>
+      <c r="I45" s="9"/>
+      <c r="J45" s="9"/>
+      <c r="K45" s="9"/>
+      <c r="L45" s="9"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="s">
@@ -4442,46 +3677,16 @@
       <c r="B46" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C46" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),17)</f>
-        <v>17</v>
-      </c>
-      <c r="D46" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),53.36)</f>
-        <v>53.36</v>
-      </c>
-      <c r="E46" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),91.52)</f>
-        <v>91.52</v>
-      </c>
-      <c r="F46" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),150.4)</f>
-        <v>150.4</v>
-      </c>
-      <c r="G46" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),152.44)</f>
-        <v>152.44</v>
-      </c>
-      <c r="H46" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),171.76)</f>
-        <v>171.76</v>
-      </c>
-      <c r="I46" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),150.8)</f>
-        <v>150.8</v>
-      </c>
-      <c r="J46" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),125.28)</f>
-        <v>125.28</v>
-      </c>
-      <c r="K46" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),117.04)</f>
-        <v>117.04</v>
-      </c>
-      <c r="L46" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),122.68)</f>
-        <v>122.68</v>
-      </c>
+      <c r="C46" s="9"/>
+      <c r="D46" s="9"/>
+      <c r="E46" s="9"/>
+      <c r="F46" s="9"/>
+      <c r="G46" s="9"/>
+      <c r="H46" s="9"/>
+      <c r="I46" s="9"/>
+      <c r="J46" s="9"/>
+      <c r="K46" s="9"/>
+      <c r="L46" s="9"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="6" t="s">
@@ -4490,46 +3695,16 @@
       <c r="B47" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C47" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2)</f>
-        <v>2</v>
-      </c>
-      <c r="D47" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.16)</f>
-        <v>3.16</v>
-      </c>
-      <c r="E47" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.4)</f>
-        <v>5.4</v>
-      </c>
-      <c r="F47" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),9.8)</f>
-        <v>9.8</v>
-      </c>
-      <c r="G47" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),9.52)</f>
-        <v>9.52</v>
-      </c>
-      <c r="H47" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),11.16)</f>
-        <v>11.16</v>
-      </c>
-      <c r="I47" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),8.88)</f>
-        <v>8.88</v>
-      </c>
-      <c r="J47" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.36)</f>
-        <v>7.36</v>
-      </c>
-      <c r="K47" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.68)</f>
-        <v>7.68</v>
-      </c>
-      <c r="L47" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7)</f>
-        <v>7</v>
-      </c>
+      <c r="C47" s="9"/>
+      <c r="D47" s="9"/>
+      <c r="E47" s="9"/>
+      <c r="F47" s="9"/>
+      <c r="G47" s="9"/>
+      <c r="H47" s="9"/>
+      <c r="I47" s="9"/>
+      <c r="J47" s="9"/>
+      <c r="K47" s="9"/>
+      <c r="L47" s="9"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="6" t="s">
@@ -4542,42 +3717,15 @@
         <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(Links!$B$5,""sobrestock_sustitutos!B86:K89"")"),1)</f>
         <v>1</v>
       </c>
-      <c r="D48" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.08)</f>
-        <v>0.08</v>
-      </c>
-      <c r="E48" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.08)</f>
-        <v>1.08</v>
-      </c>
-      <c r="F48" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.16)</f>
-        <v>1.16</v>
-      </c>
-      <c r="G48" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.24)</f>
-        <v>2.24</v>
-      </c>
-      <c r="H48" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.4)</f>
-        <v>1.4</v>
-      </c>
-      <c r="I48" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.48)</f>
-        <v>1.48</v>
-      </c>
-      <c r="J48" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.56)</f>
-        <v>1.56</v>
-      </c>
-      <c r="K48" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.64)</f>
-        <v>0.64</v>
-      </c>
-      <c r="L48" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.64)</f>
-        <v>1.64</v>
-      </c>
+      <c r="D48" s="9"/>
+      <c r="E48" s="9"/>
+      <c r="F48" s="9"/>
+      <c r="G48" s="9"/>
+      <c r="H48" s="9"/>
+      <c r="I48" s="9"/>
+      <c r="J48" s="9"/>
+      <c r="K48" s="9"/>
+      <c r="L48" s="9"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="s">
@@ -4586,46 +3734,16 @@
       <c r="B49" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C49" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1)</f>
-        <v>1</v>
-      </c>
-      <c r="D49" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.08)</f>
-        <v>1.08</v>
-      </c>
-      <c r="E49" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.16)</f>
-        <v>2.16</v>
-      </c>
-      <c r="F49" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.32)</f>
-        <v>3.32</v>
-      </c>
-      <c r="G49" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.56)</f>
-        <v>3.56</v>
-      </c>
-      <c r="H49" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.8)</f>
-        <v>3.8</v>
-      </c>
-      <c r="I49" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.04)</f>
-        <v>3.04</v>
-      </c>
-      <c r="J49" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.2)</f>
-        <v>3.2</v>
-      </c>
-      <c r="K49" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.36)</f>
-        <v>2.36</v>
-      </c>
-      <c r="L49" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.44)</f>
-        <v>2.44</v>
-      </c>
+      <c r="C49" s="9"/>
+      <c r="D49" s="9"/>
+      <c r="E49" s="9"/>
+      <c r="F49" s="9"/>
+      <c r="G49" s="9"/>
+      <c r="H49" s="9"/>
+      <c r="I49" s="9"/>
+      <c r="J49" s="9"/>
+      <c r="K49" s="9"/>
+      <c r="L49" s="9"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="s">
@@ -4634,46 +3752,16 @@
       <c r="B50" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C50" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1)</f>
-        <v>1</v>
-      </c>
-      <c r="D50" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.08)</f>
-        <v>0.08</v>
-      </c>
-      <c r="E50" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.08)</f>
-        <v>0.08</v>
-      </c>
-      <c r="F50" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.08)</f>
-        <v>1.08</v>
-      </c>
-      <c r="G50" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.16)</f>
-        <v>1.16</v>
-      </c>
-      <c r="H50" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.24)</f>
-        <v>0.24</v>
-      </c>
-      <c r="I50" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.24)</f>
-        <v>1.24</v>
-      </c>
-      <c r="J50" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.32)</f>
-        <v>0.32</v>
-      </c>
-      <c r="K50" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.32)</f>
-        <v>0.32</v>
-      </c>
-      <c r="L50" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.32)</f>
-        <v>1.32</v>
-      </c>
+      <c r="C50" s="9"/>
+      <c r="D50" s="9"/>
+      <c r="E50" s="9"/>
+      <c r="F50" s="9"/>
+      <c r="G50" s="9"/>
+      <c r="H50" s="9"/>
+      <c r="I50" s="9"/>
+      <c r="J50" s="9"/>
+      <c r="K50" s="9"/>
+      <c r="L50" s="9"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="6" t="s">
@@ -4682,46 +3770,16 @@
       <c r="B51" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C51" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1)</f>
-        <v>1</v>
-      </c>
-      <c r="D51" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.08)</f>
-        <v>0.08</v>
-      </c>
-      <c r="E51" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.08)</f>
-        <v>0.08</v>
-      </c>
-      <c r="F51" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.08)</f>
-        <v>0.08</v>
-      </c>
-      <c r="G51" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.08)</f>
-        <v>1.08</v>
-      </c>
-      <c r="H51" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.16)</f>
-        <v>0.16</v>
-      </c>
-      <c r="I51" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.16)</f>
-        <v>1.16</v>
-      </c>
-      <c r="J51" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.24)</f>
-        <v>0.24</v>
-      </c>
-      <c r="K51" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.24)</f>
-        <v>0.24</v>
-      </c>
-      <c r="L51" s="9" t="n">
-        <f aca="false">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.24)</f>
-        <v>0.24</v>
-      </c>
+      <c r="C51" s="9"/>
+      <c r="D51" s="9"/>
+      <c r="E51" s="9"/>
+      <c r="F51" s="9"/>
+      <c r="G51" s="9"/>
+      <c r="H51" s="9"/>
+      <c r="I51" s="9"/>
+      <c r="J51" s="9"/>
+      <c r="K51" s="9"/>
+      <c r="L51" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>